<commit_message>
Premahwane na teksta ot siwite kletki
</commit_message>
<xml_diff>
--- a/artefakti/s04-ocenkarisk/Шаблон - час 4 Оценка на риска (1).xlsx
+++ b/artefakti/s04-ocenkarisk/Шаблон - час 4 Оценка на риска (1).xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\borkonora\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\borkonora\Desktop\laboratorii\artefakti\s04-ocenkarisk\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8904" tabRatio="500" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8904" tabRatio="500" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Инструкции" sheetId="1" r:id="rId1"/>
@@ -102,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="287">
   <si>
     <t>МИС — инструмент за риска (инвентаризация, оценка на риска, план за третиране)</t>
   </si>
@@ -392,9 +392,6 @@
     <t>поверителна</t>
   </si>
   <si>
-    <t>◄ ПРИМЕР — замени с активите на твоята фирма</t>
-  </si>
-  <si>
     <t>A-02</t>
   </si>
   <si>
@@ -407,9 +404,6 @@
     <t>—</t>
   </si>
   <si>
-    <t>◄ ПРИМЕР</t>
-  </si>
-  <si>
     <t>A-03</t>
   </si>
   <si>
@@ -419,15 +413,9 @@
     <t>A-07</t>
   </si>
   <si>
-    <t>◄ ПРИМЕР — лични данни</t>
-  </si>
-  <si>
     <t>хардуер</t>
   </si>
   <si>
-    <t>◄ ПРИМЕР — свързан с R-04</t>
-  </si>
-  <si>
     <t>A-11</t>
   </si>
   <si>
@@ -438,9 +426,6 @@
   </si>
   <si>
     <t>Управител</t>
-  </si>
-  <si>
-    <t>◄ ПРИМЕР — знанието е актив</t>
   </si>
   <si>
     <t>R-ID</t>
@@ -2781,7 +2766,7 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
@@ -2814,7 +2799,7 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
@@ -2827,7 +2812,7 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
@@ -2837,7 +2822,7 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
@@ -3189,65 +3174,61 @@
         <v>91</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="C2" s="16" t="s">
         <v>92</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="F2" s="16" t="s">
         <v>95</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="H2" s="16" t="s">
-        <v>162</v>
-      </c>
-      <c r="I2" s="17" t="s">
-        <v>96</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="I2" s="17"/>
     </row>
     <row r="3" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C3" s="16" t="s">
         <v>92</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="F3" s="16" t="s">
         <v>95</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="I3" s="17" t="s">
-        <v>101</v>
-      </c>
+        <v>160</v>
+      </c>
+      <c r="I3" s="17"/>
     </row>
     <row r="4" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C4" s="16" t="s">
         <v>92</v>
@@ -3262,53 +3243,49 @@
         <v>95</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="I4" s="17" t="s">
-        <v>105</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="I4" s="17"/>
     </row>
     <row r="5" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="F5" s="16" t="s">
         <v>95</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="H5" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="I5" s="17" t="s">
-        <v>107</v>
-      </c>
+      <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>93</v>
@@ -3317,112 +3294,106 @@
         <v>94</v>
       </c>
       <c r="F6" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="H6" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="G6" s="16" t="s">
-        <v>174</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="I6" s="17" t="s">
-        <v>101</v>
-      </c>
+      <c r="I6" s="17"/>
     </row>
     <row r="7" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>179</v>
-      </c>
-      <c r="I7" s="17" t="s">
-        <v>112</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="I7" s="17"/>
     </row>
     <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>179</v>
-      </c>
-      <c r="I8" s="17" t="s">
-        <v>101</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="I8" s="17"/>
     </row>
     <row r="9" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="I9" s="16"/>
     </row>
     <row r="10" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D10" s="16" t="s">
         <v>93</v>
@@ -3431,22 +3402,22 @@
         <v>94</v>
       </c>
       <c r="F10" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="H10" s="16" t="s">
         <v>99</v>
-      </c>
-      <c r="G10" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="H10" s="16" t="s">
-        <v>100</v>
       </c>
       <c r="I10" s="16"/>
     </row>
     <row r="11" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>92</v>
@@ -3461,91 +3432,91 @@
         <v>95</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I11" s="16"/>
     </row>
     <row r="12" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I12" s="16"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F13" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="H13" s="16" t="s">
         <v>99</v>
-      </c>
-      <c r="G13" s="16" t="s">
-        <v>196</v>
-      </c>
-      <c r="H13" s="16" t="s">
-        <v>100</v>
       </c>
       <c r="I13" s="16"/>
     </row>
     <row r="14" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="16" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>92</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="F14" s="16" t="s">
         <v>95</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I14" s="16"/>
     </row>
@@ -5724,81 +5695,81 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B1" s="15" t="s">
         <v>82</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="I1" s="15" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="J1" s="15" t="s">
         <v>27</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="L1" s="15" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="M1" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="N1" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="O1" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="P1" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q1" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="R1" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="S1" s="15" t="s">
         <v>121</v>
-      </c>
-      <c r="O1" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="P1" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q1" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="R1" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="S1" s="15" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="66" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="F2" s="16" t="s">
         <v>199</v>
-      </c>
-      <c r="B2" s="16" t="s">
-        <v>200</v>
-      </c>
-      <c r="C2" s="16" t="s">
-        <v>201</v>
-      </c>
-      <c r="D2" s="16" t="s">
-        <v>202</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>203</v>
-      </c>
-      <c r="F2" s="16" t="s">
-        <v>204</v>
       </c>
       <c r="G2" s="16">
         <v>4</v>
@@ -5819,16 +5790,16 @@
         <v>не</v>
       </c>
       <c r="L2" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="M2" s="16" t="s">
         <v>93</v>
       </c>
       <c r="N2" s="16" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="O2" s="16" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="P2" s="16">
         <v>2</v>
@@ -5841,27 +5812,27 @@
         <v>8</v>
       </c>
       <c r="S2" s="17" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="66" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="F3" s="16" t="s">
         <v>205</v>
-      </c>
-      <c r="B3" s="16" t="s">
-        <v>206</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>207</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>209</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>210</v>
       </c>
       <c r="G3" s="16">
         <v>3</v>
@@ -5882,16 +5853,16 @@
         <v>не</v>
       </c>
       <c r="L3" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="N3" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O3" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P3" s="16">
         <v>2</v>
@@ -5904,27 +5875,27 @@
         <v>4</v>
       </c>
       <c r="S3" s="17" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="F4" s="16" t="s">
         <v>211</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>212</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>213</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>215</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>216</v>
       </c>
       <c r="G4" s="16">
         <v>2</v>
@@ -5945,10 +5916,10 @@
         <v>не</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="M4" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="N4" s="16"/>
       <c r="O4" s="16"/>
@@ -5962,22 +5933,22 @@
     </row>
     <row r="5" spans="1:19" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="G5" s="16">
         <v>4</v>
@@ -5998,10 +5969,10 @@
         <v>не</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="M5" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="N5" s="16"/>
       <c r="O5" s="16"/>
@@ -6015,22 +5986,22 @@
     </row>
     <row r="6" spans="1:19" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>219</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="F6" s="16" t="s">
         <v>222</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>223</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>224</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>225</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>226</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>227</v>
       </c>
       <c r="G6" s="16">
         <v>2</v>
@@ -6051,10 +6022,10 @@
         <v>не</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="N6" s="16"/>
       <c r="O6" s="16"/>
@@ -6068,22 +6039,22 @@
     </row>
     <row r="7" spans="1:19" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="F7" s="16" t="s">
         <v>228</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>229</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>230</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>231</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>232</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>233</v>
       </c>
       <c r="G7" s="16">
         <v>3</v>
@@ -6104,10 +6075,10 @@
         <v>не</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="N7" s="16"/>
       <c r="O7" s="16"/>
@@ -6121,22 +6092,22 @@
     </row>
     <row r="8" spans="1:19" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="G8" s="16">
         <v>3</v>
@@ -6157,10 +6128,10 @@
         <v>да</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="N8" s="16"/>
       <c r="O8" s="16"/>
@@ -6174,22 +6145,22 @@
     </row>
     <row r="9" spans="1:19" ht="66" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>237</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>238</v>
+      </c>
+      <c r="F9" s="16" t="s">
         <v>239</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>240</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>241</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>242</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>243</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>244</v>
       </c>
       <c r="G9" s="16">
         <v>3</v>
@@ -6210,10 +6181,10 @@
         <v>да</v>
       </c>
       <c r="L9" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="N9" s="16"/>
       <c r="O9" s="16"/>
@@ -6227,22 +6198,22 @@
     </row>
     <row r="10" spans="1:19" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
+        <v>240</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>244</v>
+      </c>
+      <c r="F10" s="16" t="s">
         <v>245</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>247</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>248</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>249</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>250</v>
       </c>
       <c r="G10" s="16">
         <v>1</v>
@@ -6263,10 +6234,10 @@
         <v>да</v>
       </c>
       <c r="L10" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="N10" s="16"/>
       <c r="O10" s="16"/>
@@ -6280,22 +6251,22 @@
     </row>
     <row r="11" spans="1:19" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G11" s="16">
         <v>4</v>
@@ -6316,7 +6287,7 @@
         <v>не</v>
       </c>
       <c r="L11" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="M11" s="16" t="s">
         <v>94</v>
@@ -6333,22 +6304,22 @@
     </row>
     <row r="12" spans="1:19" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>251</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>253</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>254</v>
+      </c>
+      <c r="F12" s="16" t="s">
         <v>255</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>256</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>257</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>258</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>259</v>
-      </c>
-      <c r="F12" s="16" t="s">
-        <v>260</v>
       </c>
       <c r="G12" s="16">
         <v>2</v>
@@ -6369,7 +6340,7 @@
         <v>да</v>
       </c>
       <c r="L12" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="M12" s="16" t="s">
         <v>93</v>
@@ -6386,22 +6357,22 @@
     </row>
     <row r="13" spans="1:19" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>257</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>258</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>259</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>260</v>
+      </c>
+      <c r="F13" s="16" t="s">
         <v>261</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>262</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>263</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>264</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>265</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>266</v>
       </c>
       <c r="G13" s="16">
         <v>2</v>
@@ -6422,7 +6393,7 @@
         <v>да</v>
       </c>
       <c r="L13" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="M13" s="16" t="s">
         <v>93</v>
@@ -6447,11 +6418,11 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="18" t="str">
-        <f t="shared" ref="I2:I65" si="3">IF(OR(G14="",H14=""),"",G14*H14)</f>
+        <f t="shared" ref="I14:I65" si="3">IF(OR(G14="",H14=""),"",G14*H14)</f>
         <v/>
       </c>
       <c r="J14" s="19" t="str">
-        <f t="shared" ref="J2:J65" si="4">IF(I14="","",IF(I14&lt;=4,"нисък",IF(I14&lt;=9,"умерен",IF(I14&lt;=15,"висок","критичен"))))</f>
+        <f t="shared" ref="J14:J65" si="4">IF(I14="","",IF(I14&lt;=4,"нисък",IF(I14&lt;=9,"умерен",IF(I14&lt;=15,"висок","критичен"))))</f>
         <v/>
       </c>
       <c r="K14" s="19" t="str">
@@ -12871,19 +12842,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:I13">
-    <cfRule type="cellIs" dxfId="7" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="15" priority="1" operator="between">
       <formula>1</formula>
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="14" priority="2" operator="between">
       <formula>5</formula>
       <formula>9</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="13" priority="3" operator="between">
       <formula>10</formula>
       <formula>15</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="between">
+    <cfRule type="cellIs" dxfId="12" priority="4" operator="between">
       <formula>16</formula>
       <formula>25</formula>
     </cfRule>
@@ -12925,85 +12896,85 @@
   <sheetData>
     <row r="1" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B1" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G1" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="H1" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="J1" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="K1" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="L1" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="M1" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="N1" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="O1" s="15" t="s">
         <v>138</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="G1" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="H1" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="I1" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="J1" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="K1" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="L1" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="M1" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="N1" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="O1" s="15" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="D2" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A2,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>16</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="H2" s="16" t="s">
         <v>93</v>
       </c>
       <c r="I2" s="16" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="J2" s="16" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="L2" s="16">
         <v>2</v>
@@ -13016,43 +12987,43 @@
         <v>8</v>
       </c>
       <c r="O2" s="17" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B3" s="16" t="s">
         <v>91</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D3" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A3,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>12</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="I3" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J3" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K3" s="16" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="L3" s="16">
         <v>2</v>
@@ -13065,34 +13036,34 @@
         <v>4</v>
       </c>
       <c r="O3" s="17" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="D4" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A4,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>10</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="I4" s="16"/>
       <c r="J4" s="16"/>
@@ -13107,29 +13078,29 @@
     </row>
     <row r="5" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="D5" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A5,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>12</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="I5" s="16"/>
       <c r="J5" s="16"/>
@@ -13144,29 +13115,29 @@
     </row>
     <row r="6" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="D6" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A6,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>10</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="I6" s="16"/>
       <c r="J6" s="16"/>
@@ -13181,29 +13152,29 @@
     </row>
     <row r="7" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="D7" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A7,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>12</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="I7" s="16"/>
       <c r="J7" s="16"/>
@@ -13218,29 +13189,29 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="D8" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A8,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>6</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="I8" s="16"/>
       <c r="J8" s="16"/>
@@ -13255,29 +13226,29 @@
     </row>
     <row r="9" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="D9" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A9,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>9</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="16"/>
@@ -13292,29 +13263,29 @@
     </row>
     <row r="10" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="D10" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A10,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>3</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="I10" s="16"/>
       <c r="J10" s="16"/>
@@ -13329,26 +13300,26 @@
     </row>
     <row r="11" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B11" s="16" t="s">
         <v>91</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="D11" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A11,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>12</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="H11" s="16" t="s">
         <v>94</v>
@@ -13366,26 +13337,26 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="D12" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A12,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>6</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H12" s="16" t="s">
         <v>93</v>
@@ -13403,26 +13374,26 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="D13" s="19">
         <f>IFERROR(INDEX('[1]Регистър на риска'!$I:$I,MATCH(A13,'[1]Регистър на риска'!$A:$A,0)),"")</f>
         <v>4</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H13" s="16" t="s">
         <v>93</v>
@@ -17880,37 +17851,37 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D14:D210">
-    <cfRule type="cellIs" dxfId="15" priority="6" operator="between">
+    <cfRule type="cellIs" dxfId="11" priority="6" operator="between">
       <formula>1</formula>
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="7" operator="between">
+    <cfRule type="cellIs" dxfId="10" priority="7" operator="between">
       <formula>5</formula>
       <formula>9</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="8" operator="between">
+    <cfRule type="cellIs" dxfId="9" priority="8" operator="between">
       <formula>10</formula>
       <formula>15</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="9" operator="between">
+    <cfRule type="cellIs" dxfId="8" priority="9" operator="between">
       <formula>16</formula>
       <formula>25</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N210">
-    <cfRule type="cellIs" dxfId="11" priority="10" operator="between">
+    <cfRule type="cellIs" dxfId="7" priority="10" operator="between">
       <formula>1</formula>
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="11" operator="between">
+    <cfRule type="cellIs" dxfId="6" priority="11" operator="between">
       <formula>5</formula>
       <formula>9</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="12" operator="between">
+    <cfRule type="cellIs" dxfId="5" priority="12" operator="between">
       <formula>10</formula>
       <formula>15</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="13" operator="between">
+    <cfRule type="cellIs" dxfId="4" priority="13" operator="between">
       <formula>16</formula>
       <formula>25</formula>
     </cfRule>

</xml_diff>